<commit_message>
Bump dates and begin updates
</commit_message>
<xml_diff>
--- a/data/data_sources.xlsx
+++ b/data/data_sources.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10811"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kjhealy/Documents/courses/mptc/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C765BCE-3944-EA44-B67B-784632640A5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66A251FC-2826-C440-B7F4-2A125D275A74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="540" yWindow="1660" windowWidth="33540" windowHeight="16460" xr2:uid="{FF444104-2C96-9340-A7A7-D0D5BB267F7C}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
   <si>
     <t>name</t>
   </si>
@@ -112,6 +112,24 @@
   </si>
   <si>
     <t>https://kjhealy.github.io/gssr/</t>
+  </si>
+  <si>
+    <t>American National Election Study (ANES)</t>
+  </si>
+  <si>
+    <t>https://electionstudies.org</t>
+  </si>
+  <si>
+    <t>Eurostat</t>
+  </si>
+  <si>
+    <t>https://ec.europa.eu/eurostat</t>
+  </si>
+  <si>
+    <t>Project Gutenberg</t>
+  </si>
+  <si>
+    <t>https://www.gutenberg.org</t>
   </si>
 </sst>
 </file>
@@ -469,7 +487,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71FE4373-BD3B-FD48-B504-CA3F219CBEF5}">
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="62" customWidth="1"/>
@@ -579,6 +597,30 @@
         <v>25</v>
       </c>
     </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>28</v>
+      </c>
+      <c r="B15" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" t="s">
+        <v>31</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>